<commit_message>
generate_example_sheets work - next step incorporate descriptions
</commit_message>
<xml_diff>
--- a/static/example_sheets/CGG Animal Plant.xlsx
+++ b/static/example_sheets/CGG Animal Plant.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\magnu\Documents\Git Repoes\gg-metadatabase-ui\static\example_sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glj523\Documents\github repoes\upload_web_app\static\example_sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF4D5B7-F2D6-4891-8FBA-977EAAB22A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE65EA2-C0B1-4043-B301-314012E06417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
   </bookViews>
   <sheets>
     <sheet name="eDNA_Archive_sampling_(20231027" sheetId="2" r:id="rId1"/>
@@ -1896,7 +1896,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1931,12 +1931,11 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5"/>
@@ -1944,7 +1943,7 @@
   <cellStyles count="8">
     <cellStyle name="Comma 2" xfId="3" xr:uid="{8942F21F-F0D4-468F-A2D9-2DD07A9F09D0}"/>
     <cellStyle name="Explanatory Text 2" xfId="2" xr:uid="{EEC8BC1F-FCCB-4C2D-96AE-E4673B111AFF}"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{C43A14CE-CD9A-4CDB-8396-19B2B1DC1FD5}"/>
     <cellStyle name="Normal 4" xfId="4" xr:uid="{1133FEEC-7998-4312-B355-8FD805FAFB7D}"/>
@@ -2246,9 +2245,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022 Tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2286,7 +2285,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2392,7 +2391,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2534,7 +2533,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2597,171 +2596,171 @@
     <col min="50" max="50" width="13.77734375" customWidth="1"/>
     <col min="51" max="51" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="100.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="29.109375" customWidth="1"/>
     <col min="54" max="54" width="19.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" s="18" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:54" s="17" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="L1" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="M1" s="18" t="s">
+      <c r="M1" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="N1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="O1" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="P1" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="Q1" s="18" t="s">
+      <c r="Q1" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="R1" s="18" t="s">
+      <c r="R1" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="S1" s="18" t="s">
+      <c r="S1" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="18" t="s">
+      <c r="T1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="U1" s="18" t="s">
+      <c r="U1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="V1" s="18" t="s">
+      <c r="V1" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="W1" s="18" t="s">
+      <c r="W1" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="X1" s="18" t="s">
+      <c r="X1" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="Y1" s="18" t="s">
+      <c r="Y1" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="Z1" s="18" t="s">
+      <c r="Z1" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="AA1" s="18" t="s">
+      <c r="AA1" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="AB1" s="18" t="s">
+      <c r="AB1" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="AC1" s="18" t="s">
+      <c r="AC1" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="AD1" s="18" t="s">
+      <c r="AD1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="AE1" s="18" t="s">
+      <c r="AE1" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="AF1" s="18" t="s">
+      <c r="AF1" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="AG1" s="18" t="s">
+      <c r="AG1" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="AH1" s="18" t="s">
+      <c r="AH1" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="AI1" s="18" t="s">
+      <c r="AI1" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="AJ1" s="18" t="s">
+      <c r="AJ1" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="AK1" s="18" t="s">
+      <c r="AK1" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="AL1" s="18" t="s">
+      <c r="AL1" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="AM1" s="18" t="s">
+      <c r="AM1" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="AN1" s="18" t="s">
+      <c r="AN1" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="AO1" s="18" t="s">
+      <c r="AO1" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="AP1" s="18" t="s">
+      <c r="AP1" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="AQ1" s="18" t="s">
+      <c r="AQ1" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AR1" s="18" t="s">
+      <c r="AR1" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="AS1" s="18" t="s">
+      <c r="AS1" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="AT1" s="18" t="s">
+      <c r="AT1" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="AU1" s="18" t="s">
+      <c r="AU1" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="AV1" s="18" t="s">
+      <c r="AV1" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="AW1" s="18" t="s">
+      <c r="AW1" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="AX1" s="18" t="s">
+      <c r="AX1" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="AY1" s="18" t="s">
+      <c r="AY1" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="AZ1" s="18" t="s">
+      <c r="AZ1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="BA1" s="18" t="s">
+      <c r="BA1" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="BB1" s="18" t="s">
+      <c r="BB1" s="17" t="s">
         <v>41</v>
       </c>
     </row>
@@ -2850,10 +2849,7 @@
       <c r="AV2" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="AY2" s="14"/>
-      <c r="AZ2" s="15"/>
-      <c r="BA2" s="14"/>
-      <c r="BB2" s="14"/>
+      <c r="AZ2" s="14"/>
     </row>
     <row r="3" spans="1:54" s="11" customFormat="1" ht="12.6" x14ac:dyDescent="0.2">
       <c r="B3" s="8" t="s">
@@ -2946,12 +2942,9 @@
       <c r="AV3" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="AY3" s="14"/>
-      <c r="AZ3" s="14" t="s">
+      <c r="AZ3" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="BA3" s="14"/>
-      <c r="BB3" s="14"/>
     </row>
     <row r="4" spans="1:54" s="11" customFormat="1" ht="12.6" x14ac:dyDescent="0.2">
       <c r="B4" s="8" t="s">
@@ -3044,12 +3037,9 @@
       <c r="AV4" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="AY4" s="14"/>
-      <c r="AZ4" s="14" t="s">
+      <c r="AZ4" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="BA4" s="14"/>
-      <c r="BB4" s="14"/>
     </row>
     <row r="5" spans="1:54" s="1" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
@@ -3097,20 +3087,20 @@
       <c r="AT5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="AY5" s="16"/>
-      <c r="AZ5" s="16"/>
-      <c r="BA5" s="16"/>
-      <c r="BB5" s="16"/>
+      <c r="AY5" s="15"/>
+      <c r="AZ5" s="15"/>
+      <c r="BA5" s="15"/>
+      <c r="BB5" s="15"/>
     </row>
     <row r="6" spans="1:54" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
       <c r="AD6" s="4"/>
-      <c r="AY6" s="17"/>
-      <c r="AZ6" s="17"/>
-      <c r="BA6" s="17"/>
-      <c r="BB6" s="17"/>
+      <c r="AY6" s="16"/>
+      <c r="AZ6" s="16"/>
+      <c r="BA6" s="16"/>
+      <c r="BB6" s="16"/>
     </row>
     <row r="7" spans="1:54" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -3141,10 +3131,10 @@
       <c r="AJ7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="AY7" s="17"/>
-      <c r="AZ7" s="17"/>
-      <c r="BA7" s="17"/>
-      <c r="BB7" s="17"/>
+      <c r="AY7" s="16"/>
+      <c r="AZ7" s="16"/>
+      <c r="BA7" s="16"/>
+      <c r="BB7" s="16"/>
     </row>
     <row r="8" spans="1:54" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
@@ -3162,10 +3152,10 @@
       <c r="S8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="AY8" s="16"/>
-      <c r="AZ8" s="16"/>
-      <c r="BA8" s="16"/>
-      <c r="BB8" s="16"/>
+      <c r="AY8" s="15"/>
+      <c r="AZ8" s="15"/>
+      <c r="BA8" s="15"/>
+      <c r="BB8" s="15"/>
     </row>
     <row r="11" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -3175,35 +3165,8 @@
     <row r="19" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="19" type="noConversion"/>
-  <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="E1:E4" xr:uid="{C3D5741D-363E-4A57-92ED-A7C1AF363103}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="AR1:AR4" xr:uid="{4E1E3514-9597-4937-9B82-3064EC2A28DB}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="BB1 AQ1:AQ4" xr:uid="{9433CAC5-14C8-4BC5-98F4-9DCC500EB689}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="AB1:AB4" xr:uid="{0A1292F7-D57C-4D23-9F2E-A42A608617CE}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="T1:T4" xr:uid="{70051D4A-C1E3-42EB-AB75-69159BBA6EE6}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="S1:S4" xr:uid="{6517AB40-F657-43A7-93C5-01939C7B30A3}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="Q1:Q4" xr:uid="{D7B1F3B7-57F8-48DB-A858-D07EFD9240E1}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="M1:M4" xr:uid="{5011E372-B897-44AA-800A-6311525028B0}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="L1:L4" xr:uid="{2F750084-D97F-4E4E-B24D-67C7807BD2CA}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="BA1:BA4" xr:uid="{78A7C043-50A7-4709-82EC-A9A4EDACB525}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="E1:E4 BA1:BA4 L1:M4 Q1:Q4 S1:T4 AB1:AB4 BB1 AQ1:AR4" xr:uid="{C3D5741D-363E-4A57-92ED-A7C1AF363103}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>